<commit_message>
Stationen und Gelingensnachweis aus den Bausteinuebersichten (Jg5/6/7)
416 Stationen in 33 Bausteinen aus den WORD-Uebersichten eingetragen
(Pflicht/Wahl und Schwierigkeit aus den Grafiken der Dokumente).
Jg7-Wahlstationen mit Gymnasiasten-Hinweis. Offen: Jg6 DE 3 (zwei
Lektuere-Alternativen), Jg7 BIO 2-4 (Dokument ohne Titel), Mathe Jg6.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/jahrgaenge/Jg7.xlsx
+++ b/content/jahrgaenge/Jg7.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2107" uniqueCount="443">
   <si>
     <t>Hinweise zu Jg7.xlsx</t>
   </si>
@@ -616,6 +616,18 @@
     <t>Fallbericht an das Gesundheitsamt</t>
   </si>
   <si>
+    <t>The Magic Mirror</t>
+  </si>
+  <si>
+    <t>design a reading journal</t>
+  </si>
+  <si>
+    <t>Orientierung auf der Erde</t>
+  </si>
+  <si>
+    <t>Anwenden des erlernten Wissens, um das ausgefallene Navigationssystem neu zu starten</t>
+  </si>
+  <si>
     <t>Die geheimnisvolle Welt der Balladen</t>
   </si>
   <si>
@@ -854,6 +866,159 @@
   </si>
   <si>
     <t>Läuft über 2 Termine à 90 Minuten.</t>
+  </si>
+  <si>
+    <t>What's a magic mirror?</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>Judging a Book by Its Cover</t>
+  </si>
+  <si>
+    <t>your book</t>
+  </si>
+  <si>
+    <t>Getting Started: How to Team Reader (2.1)</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>Getting Started: My Reading Journal (2.2)</t>
+  </si>
+  <si>
+    <t>The first part of the story</t>
+  </si>
+  <si>
+    <t>a laptop, A3</t>
+  </si>
+  <si>
+    <t>In the museum (4.1)</t>
+  </si>
+  <si>
+    <t>A4, A5</t>
+  </si>
+  <si>
+    <t>Museums (4.2)</t>
+  </si>
+  <si>
+    <t>a laptop</t>
+  </si>
+  <si>
+    <t>Travelling back in time – Ruby</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>Travelling back in time – Noah</t>
+  </si>
+  <si>
+    <t>A7</t>
+  </si>
+  <si>
+    <t>Travelling back in time – Layla</t>
+  </si>
+  <si>
+    <t>A8</t>
+  </si>
+  <si>
+    <t>In the Tower</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>Run, Ruby, Run!</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>Visiting the market</t>
+  </si>
+  <si>
+    <t>A11</t>
+  </si>
+  <si>
+    <t>Medieval markets (10.1)</t>
+  </si>
+  <si>
+    <t>How to defeat the Spanish</t>
+  </si>
+  <si>
+    <t>A12</t>
+  </si>
+  <si>
+    <t>Getting back with a surprise</t>
+  </si>
+  <si>
+    <t>A13 / A 14 / A15</t>
+  </si>
+  <si>
+    <t>Leaving the Magic Mirror behind</t>
+  </si>
+  <si>
+    <t>A16 / A17 / A18, M4, M5</t>
+  </si>
+  <si>
+    <t>Das Gradnetz der Erde</t>
+  </si>
+  <si>
+    <t>M1 &amp; 2, A1 &amp; 2, Atlas</t>
+  </si>
+  <si>
+    <t>Geographische Koordinaten</t>
+  </si>
+  <si>
+    <t>M3, A3–6, Atlas</t>
+  </si>
+  <si>
+    <t>Wie weiß mein Handy, wo ich bin?</t>
+  </si>
+  <si>
+    <t>M4, A7, Atlas</t>
+  </si>
+  <si>
+    <t>Zeitzonen der Erde</t>
+  </si>
+  <si>
+    <t>M5, A8–11, Atlas</t>
+  </si>
+  <si>
+    <t>Beleuchtungszonen der Erde</t>
+  </si>
+  <si>
+    <t>A12–13, Laptop</t>
+  </si>
+  <si>
+    <t>Entstehung der Jahreszeiten</t>
+  </si>
+  <si>
+    <t>M6, A14–17</t>
+  </si>
+  <si>
+    <t>Schalenaufbau der Erde</t>
+  </si>
+  <si>
+    <t>M7, A18–19, Kleber &amp; Schere</t>
+  </si>
+  <si>
+    <t>Klimazonen und Klimadiagramme</t>
+  </si>
+  <si>
+    <t>A20–21, M8, Atlas</t>
+  </si>
+  <si>
+    <t>Warum lügen Weltkarten?</t>
+  </si>
+  <si>
+    <t>A22, Atlas</t>
+  </si>
+  <si>
+    <t>A23/0-5, Atlas</t>
   </si>
   <si>
     <t>2026-08-24</t>
@@ -3730,16 +3895,16 @@
         <v>166</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>198</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>8</v>
+        <v>199</v>
+      </c>
+      <c r="F3">
+        <v>17</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>8</v>
@@ -3756,16 +3921,16 @@
         <v>168</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>8</v>
+        <v>200</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" t="s">
-        <v>8</v>
+        <v>201</v>
+      </c>
+      <c r="F4">
+        <v>10</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>8</v>
@@ -3782,13 +3947,13 @@
         <v>44</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F5" t="s">
         <v>8</v>
@@ -3808,13 +3973,13 @@
         <v>171</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F6">
         <v>13</v>
@@ -4224,7 +4389,7 @@
         <v>193</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>8</v>
@@ -4259,7 +4424,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -4304,7 +4469,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D2" t="s">
         <v>93</v>
@@ -4316,7 +4481,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>8</v>
@@ -4330,7 +4495,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D3" t="s">
         <v>93</v>
@@ -4342,7 +4507,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>8</v>
@@ -4356,7 +4521,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="D4" t="s">
         <v>93</v>
@@ -4368,7 +4533,7 @@
         <v>2</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>8</v>
@@ -4382,7 +4547,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D5" t="s">
         <v>93</v>
@@ -4394,7 +4559,7 @@
         <v>2</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>8</v>
@@ -4408,7 +4573,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D6" t="s">
         <v>93</v>
@@ -4420,7 +4585,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>8</v>
@@ -4434,10 +4599,10 @@
         <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D7" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E7">
         <v>90</v>
@@ -4446,10 +4611,10 @@
         <v>2</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -4460,7 +4625,7 @@
         <v>7</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="D8" t="s">
         <v>93</v>
@@ -4472,7 +4637,7 @@
         <v>1</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>8</v>
@@ -4486,10 +4651,10 @@
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="D9" t="s">
         <v>215</v>
-      </c>
-      <c r="D9" t="s">
-        <v>211</v>
       </c>
       <c r="E9">
         <v>90</v>
@@ -4498,10 +4663,10 @@
         <v>2</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -4512,7 +4677,7 @@
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D10" t="s">
         <v>93</v>
@@ -4524,7 +4689,7 @@
         <v>2</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>8</v>
@@ -4538,7 +4703,7 @@
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D11" t="s">
         <v>93</v>
@@ -4550,7 +4715,7 @@
         <v>2</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>8</v>
@@ -4564,7 +4729,7 @@
         <v>11</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D12" t="s">
         <v>93</v>
@@ -4576,7 +4741,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="H12" s="2" t="s">
         <v>8</v>
@@ -4590,10 +4755,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="D13" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E13">
         <v>60</v>
@@ -4602,10 +4767,10 @@
         <v>3</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -4616,7 +4781,7 @@
         <v>13</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="D14" t="s">
         <v>93</v>
@@ -4628,7 +4793,7 @@
         <v>3</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>8</v>
@@ -4642,7 +4807,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D15" t="s">
         <v>93</v>
@@ -4654,7 +4819,7 @@
         <v>2</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H15" s="2" t="s">
         <v>8</v>
@@ -4668,7 +4833,7 @@
         <v>2</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="D16" t="s">
         <v>93</v>
@@ -4680,7 +4845,7 @@
         <v>2</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="H16" s="2" t="s">
         <v>8</v>
@@ -4694,10 +4859,10 @@
         <v>3</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="D17" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E17">
         <v>40</v>
@@ -4706,10 +4871,10 @@
         <v>3</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
@@ -4720,10 +4885,10 @@
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="D18" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E18">
         <v>40</v>
@@ -4732,10 +4897,10 @@
         <v>3</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -4746,7 +4911,7 @@
         <v>5</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D19" t="s">
         <v>93</v>
@@ -4758,7 +4923,7 @@
         <v>3</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>8</v>
@@ -4772,7 +4937,7 @@
         <v>6</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D20" t="s">
         <v>93</v>
@@ -4784,7 +4949,7 @@
         <v>3</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="H20" s="2" t="s">
         <v>8</v>
@@ -4798,7 +4963,7 @@
         <v>7</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D21" t="s">
         <v>93</v>
@@ -4810,7 +4975,7 @@
         <v>2</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>8</v>
@@ -4824,10 +4989,10 @@
         <v>8</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D22" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E22">
         <v>40</v>
@@ -4836,10 +5001,10 @@
         <v>2</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
@@ -4850,7 +5015,7 @@
         <v>9</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="D23" t="s">
         <v>93</v>
@@ -4862,7 +5027,7 @@
         <v>3</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="H23" s="2" t="s">
         <v>8</v>
@@ -4876,7 +5041,7 @@
         <v>10</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="D24" t="s">
         <v>93</v>
@@ -4888,7 +5053,7 @@
         <v>1</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H24" s="2" t="s">
         <v>8</v>
@@ -4902,10 +5067,10 @@
         <v>11</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D25" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E25">
         <v>40</v>
@@ -4914,10 +5079,10 @@
         <v>3</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -4928,7 +5093,7 @@
         <v>12</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="D26" t="s">
         <v>93</v>
@@ -4940,7 +5105,7 @@
         <v>3</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="H26" s="2" t="s">
         <v>8</v>
@@ -4954,10 +5119,10 @@
         <v>13</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D27" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E27">
         <v>30</v>
@@ -4966,10 +5131,10 @@
         <v>2</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -4980,10 +5145,10 @@
         <v>14</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="D28" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E28">
         <v>30</v>
@@ -4992,10 +5157,10 @@
         <v>2</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -5006,10 +5171,10 @@
         <v>1</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D29" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E29">
         <v>10</v>
@@ -5018,10 +5183,10 @@
         <v>1</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -5032,7 +5197,7 @@
         <v>2</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D30" t="s">
         <v>93</v>
@@ -5044,7 +5209,7 @@
         <v>2</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="H30" s="2" t="s">
         <v>8</v>
@@ -5058,7 +5223,7 @@
         <v>3</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="D31" t="s">
         <v>93</v>
@@ -5070,7 +5235,7 @@
         <v>2</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>8</v>
@@ -5084,7 +5249,7 @@
         <v>4</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="D32" t="s">
         <v>93</v>
@@ -5096,7 +5261,7 @@
         <v>3</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>8</v>
@@ -5110,7 +5275,7 @@
         <v>5</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="D33" t="s">
         <v>93</v>
@@ -5122,7 +5287,7 @@
         <v>2</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="H33" s="2" t="s">
         <v>8</v>
@@ -5136,7 +5301,7 @@
         <v>6</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="D34" t="s">
         <v>93</v>
@@ -5148,7 +5313,7 @@
         <v>3</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="H34" s="2" t="s">
         <v>8</v>
@@ -5162,7 +5327,7 @@
         <v>7</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="D35" t="s">
         <v>93</v>
@@ -5174,7 +5339,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="H35" s="2" t="s">
         <v>8</v>
@@ -5188,10 +5353,10 @@
         <v>8</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="D36" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E36">
         <v>15</v>
@@ -5200,10 +5365,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -5214,7 +5379,7 @@
         <v>9</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="D37" t="s">
         <v>93</v>
@@ -5226,7 +5391,7 @@
         <v>3</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>8</v>
@@ -5240,7 +5405,7 @@
         <v>10</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="D38" t="s">
         <v>93</v>
@@ -5252,7 +5417,7 @@
         <v>2</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>8</v>
@@ -5266,10 +5431,10 @@
         <v>11</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="D39" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E39">
         <v>10</v>
@@ -5278,10 +5443,10 @@
         <v>1</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
@@ -5292,7 +5457,7 @@
         <v>12</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="D40" t="s">
         <v>93</v>
@@ -5304,7 +5469,7 @@
         <v>2</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>8</v>
@@ -5318,10 +5483,10 @@
         <v>13</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="D41" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E41">
         <v>10</v>
@@ -5330,10 +5495,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -5344,7 +5509,7 @@
         <v>14</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="D42" t="s">
         <v>93</v>
@@ -5356,7 +5521,7 @@
         <v>2</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="H42" s="2" t="s">
         <v>8</v>
@@ -5370,10 +5535,10 @@
         <v>15</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="D43" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E43">
         <v>45</v>
@@ -5382,10 +5547,10 @@
         <v>1</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="H43" s="2" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -5396,7 +5561,7 @@
         <v>16</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="D44" t="s">
         <v>93</v>
@@ -5408,10 +5573,712 @@
         <v>3</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>277</v>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>165</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="D45" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45">
+        <v>45</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>165</v>
+      </c>
+      <c r="B46">
+        <v>2</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="D46" t="s">
+        <v>93</v>
+      </c>
+      <c r="E46">
+        <v>15</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>165</v>
+      </c>
+      <c r="B47">
+        <v>3</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="D47" t="s">
+        <v>93</v>
+      </c>
+      <c r="E47">
+        <v>20</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>165</v>
+      </c>
+      <c r="B48">
+        <v>4</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="D48" t="s">
+        <v>93</v>
+      </c>
+      <c r="E48">
+        <v>10</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>165</v>
+      </c>
+      <c r="B49">
+        <v>5</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D49" t="s">
+        <v>93</v>
+      </c>
+      <c r="E49">
+        <v>90</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>165</v>
+      </c>
+      <c r="B50">
+        <v>6</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="D50" t="s">
+        <v>93</v>
+      </c>
+      <c r="E50">
+        <v>70</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>165</v>
+      </c>
+      <c r="B51">
+        <v>7</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="D51" t="s">
+        <v>215</v>
+      </c>
+      <c r="E51">
+        <v>90</v>
+      </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>165</v>
+      </c>
+      <c r="B52">
+        <v>8</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="D52" t="s">
+        <v>93</v>
+      </c>
+      <c r="E52">
+        <v>90</v>
+      </c>
+      <c r="F52">
+        <v>2</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>165</v>
+      </c>
+      <c r="B53">
+        <v>9</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D53" t="s">
+        <v>93</v>
+      </c>
+      <c r="E53">
+        <v>90</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>165</v>
+      </c>
+      <c r="B54">
+        <v>10</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D54" t="s">
+        <v>93</v>
+      </c>
+      <c r="E54">
+        <v>90</v>
+      </c>
+      <c r="F54">
+        <v>3</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>165</v>
+      </c>
+      <c r="B55">
+        <v>11</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D55" t="s">
+        <v>93</v>
+      </c>
+      <c r="E55">
+        <v>120</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>165</v>
+      </c>
+      <c r="B56">
+        <v>12</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="D56" t="s">
+        <v>93</v>
+      </c>
+      <c r="E56">
+        <v>90</v>
+      </c>
+      <c r="F56">
+        <v>2</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>165</v>
+      </c>
+      <c r="B57">
+        <v>13</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="D57" t="s">
+        <v>93</v>
+      </c>
+      <c r="E57">
+        <v>90</v>
+      </c>
+      <c r="F57">
+        <v>1</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>165</v>
+      </c>
+      <c r="B58">
+        <v>14</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="D58" t="s">
+        <v>215</v>
+      </c>
+      <c r="E58">
+        <v>50</v>
+      </c>
+      <c r="F58">
+        <v>2</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>165</v>
+      </c>
+      <c r="B59">
+        <v>15</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D59" t="s">
+        <v>93</v>
+      </c>
+      <c r="E59">
+        <v>90</v>
+      </c>
+      <c r="F59">
+        <v>3</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>165</v>
+      </c>
+      <c r="B60">
+        <v>16</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D60" t="s">
+        <v>93</v>
+      </c>
+      <c r="E60">
+        <v>90</v>
+      </c>
+      <c r="F60">
+        <v>2</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>165</v>
+      </c>
+      <c r="B61">
+        <v>17</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D61" t="s">
+        <v>93</v>
+      </c>
+      <c r="E61">
+        <v>180</v>
+      </c>
+      <c r="F61">
+        <v>3</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>167</v>
+      </c>
+      <c r="B62">
+        <v>1</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="D62" t="s">
+        <v>93</v>
+      </c>
+      <c r="E62">
+        <v>65</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>167</v>
+      </c>
+      <c r="B63">
+        <v>2</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D63" t="s">
+        <v>93</v>
+      </c>
+      <c r="E63">
+        <v>90</v>
+      </c>
+      <c r="F63">
+        <v>2</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>167</v>
+      </c>
+      <c r="B64">
+        <v>3</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D64" t="s">
+        <v>215</v>
+      </c>
+      <c r="E64">
+        <v>20</v>
+      </c>
+      <c r="F64">
+        <v>2</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>167</v>
+      </c>
+      <c r="B65">
+        <v>4</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="D65" t="s">
+        <v>93</v>
+      </c>
+      <c r="E65">
+        <v>115</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>167</v>
+      </c>
+      <c r="B66">
+        <v>5</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="D66" t="s">
+        <v>93</v>
+      </c>
+      <c r="E66">
+        <v>40</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>323</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>167</v>
+      </c>
+      <c r="B67">
+        <v>6</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="D67" t="s">
+        <v>93</v>
+      </c>
+      <c r="E67">
+        <v>110</v>
+      </c>
+      <c r="F67">
+        <v>2</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>167</v>
+      </c>
+      <c r="B68">
+        <v>7</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="D68" t="s">
+        <v>93</v>
+      </c>
+      <c r="E68">
+        <v>50</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>167</v>
+      </c>
+      <c r="B69">
+        <v>8</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="D69" t="s">
+        <v>93</v>
+      </c>
+      <c r="E69">
+        <v>120</v>
+      </c>
+      <c r="F69">
+        <v>2</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>167</v>
+      </c>
+      <c r="B70">
+        <v>9</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="D70" t="s">
+        <v>215</v>
+      </c>
+      <c r="E70">
+        <v>30</v>
+      </c>
+      <c r="F70">
+        <v>2</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>167</v>
+      </c>
+      <c r="B71">
+        <v>10</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D71" t="s">
+        <v>93</v>
+      </c>
+      <c r="E71">
+        <v>90</v>
+      </c>
+      <c r="F71">
+        <v>2</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -5587,7 +6454,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>278</v>
+        <v>333</v>
       </c>
       <c r="B2" t="s">
         <v>138</v>
@@ -5596,7 +6463,7 @@
         <v>168</v>
       </c>
       <c r="D2" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
@@ -5605,7 +6472,7 @@
         <v>8</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>280</v>
+        <v>335</v>
       </c>
       <c r="H2" t="s">
         <v>8</v>
@@ -5619,16 +6486,16 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>278</v>
+        <v>333</v>
       </c>
       <c r="B3" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E3" t="s">
         <v>8</v>
@@ -5651,16 +6518,16 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>283</v>
+        <v>338</v>
       </c>
       <c r="B4" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
@@ -5683,7 +6550,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>285</v>
+        <v>340</v>
       </c>
       <c r="B5" t="s">
         <v>138</v>
@@ -5692,7 +6559,7 @@
         <v>166</v>
       </c>
       <c r="D5" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E5" t="s">
         <v>8</v>
@@ -5701,7 +6568,7 @@
         <v>8</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>287</v>
+        <v>342</v>
       </c>
       <c r="H5" t="s">
         <v>8</v>
@@ -5715,16 +6582,16 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>285</v>
+        <v>340</v>
       </c>
       <c r="B6" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
       </c>
       <c r="D6" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E6" t="s">
         <v>8</v>
@@ -5747,16 +6614,16 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>289</v>
+        <v>344</v>
       </c>
       <c r="B7" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
@@ -5779,7 +6646,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>291</v>
+        <v>346</v>
       </c>
       <c r="B8" t="s">
         <v>138</v>
@@ -5797,7 +6664,7 @@
         <v>8</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>292</v>
+        <v>347</v>
       </c>
       <c r="H8" t="s">
         <v>8</v>
@@ -5820,7 +6687,7 @@
         <v>168</v>
       </c>
       <c r="D9" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
@@ -5829,7 +6696,7 @@
         <v>8</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>293</v>
+        <v>348</v>
       </c>
       <c r="H9" t="s">
         <v>8</v>
@@ -5846,13 +6713,13 @@
         <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="D10" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E10" t="s">
         <v>8</v>
@@ -5875,16 +6742,16 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>294</v>
+        <v>349</v>
       </c>
       <c r="B11" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
       </c>
       <c r="D11" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E11" t="s">
         <v>8</v>
@@ -5907,7 +6774,7 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>295</v>
+        <v>350</v>
       </c>
       <c r="B12" t="s">
         <v>138</v>
@@ -5916,7 +6783,7 @@
         <v>166</v>
       </c>
       <c r="D12" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
@@ -5925,7 +6792,7 @@
         <v>8</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>296</v>
+        <v>351</v>
       </c>
       <c r="H12">
         <v>13</v>
@@ -5939,16 +6806,16 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>295</v>
+        <v>350</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C13" t="s">
         <v>8</v>
       </c>
       <c r="D13" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E13" t="s">
         <v>8</v>
@@ -5971,16 +6838,16 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>297</v>
+        <v>352</v>
       </c>
       <c r="B14" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C14" t="s">
         <v>8</v>
       </c>
       <c r="D14" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E14" t="s">
         <v>8</v>
@@ -6003,7 +6870,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>298</v>
+        <v>353</v>
       </c>
       <c r="B15" t="s">
         <v>138</v>
@@ -6021,7 +6888,7 @@
         <v>8</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>299</v>
+        <v>354</v>
       </c>
       <c r="H15" t="s">
         <v>8</v>
@@ -6035,16 +6902,16 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>298</v>
+        <v>353</v>
       </c>
       <c r="B16" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C16" t="s">
         <v>8</v>
       </c>
       <c r="D16" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E16" t="s">
         <v>8</v>
@@ -6076,7 +6943,7 @@
         <v>168</v>
       </c>
       <c r="D17" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
@@ -6085,7 +6952,7 @@
         <v>8</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>300</v>
+        <v>355</v>
       </c>
       <c r="H17" t="s">
         <v>8</v>
@@ -6102,13 +6969,13 @@
         <v>127</v>
       </c>
       <c r="B18" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C18" t="s">
         <v>8</v>
       </c>
       <c r="D18" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E18" t="s">
         <v>8</v>
@@ -6134,13 +7001,13 @@
         <v>136</v>
       </c>
       <c r="B19" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C19" t="s">
         <v>8</v>
       </c>
       <c r="D19" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E19" t="s">
         <v>8</v>
@@ -6163,7 +7030,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="B20" t="s">
         <v>138</v>
@@ -6172,7 +7039,7 @@
         <v>166</v>
       </c>
       <c r="D20" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E20" t="s">
         <v>8</v>
@@ -6181,7 +7048,7 @@
         <v>8</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>302</v>
+        <v>357</v>
       </c>
       <c r="H20">
         <v>12</v>
@@ -6195,16 +7062,16 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>301</v>
+        <v>356</v>
       </c>
       <c r="B21" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C21" t="s">
         <v>8</v>
       </c>
       <c r="D21" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E21" t="s">
         <v>8</v>
@@ -6227,16 +7094,16 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>303</v>
+        <v>358</v>
       </c>
       <c r="B22" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C22" t="s">
         <v>8</v>
       </c>
       <c r="D22" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E22" t="s">
         <v>8</v>
@@ -6259,7 +7126,7 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
       <c r="B23" t="s">
         <v>138</v>
@@ -6277,7 +7144,7 @@
         <v>8</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>305</v>
+        <v>360</v>
       </c>
       <c r="H23" t="s">
         <v>8</v>
@@ -6291,16 +7158,16 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>304</v>
+        <v>359</v>
       </c>
       <c r="B24" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
       </c>
       <c r="D24" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E24" t="s">
         <v>8</v>
@@ -6323,16 +7190,16 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>306</v>
+        <v>361</v>
       </c>
       <c r="B25" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C25" t="s">
         <v>8</v>
       </c>
       <c r="D25" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E25" t="s">
         <v>8</v>
@@ -6355,16 +7222,16 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>307</v>
+        <v>362</v>
       </c>
       <c r="B26" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C26" t="s">
         <v>8</v>
       </c>
       <c r="D26" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
@@ -6387,16 +7254,16 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>308</v>
+        <v>363</v>
       </c>
       <c r="B27" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C27" t="s">
         <v>8</v>
       </c>
       <c r="D27" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E27" t="s">
         <v>8</v>
@@ -6419,7 +7286,7 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>309</v>
+        <v>364</v>
       </c>
       <c r="B28" t="s">
         <v>138</v>
@@ -6428,7 +7295,7 @@
         <v>171</v>
       </c>
       <c r="D28" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
@@ -6451,16 +7318,16 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>311</v>
+        <v>366</v>
       </c>
       <c r="B29" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C29" t="s">
         <v>8</v>
       </c>
       <c r="D29" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E29" t="s">
         <v>8</v>
@@ -6483,7 +7350,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>312</v>
+        <v>367</v>
       </c>
       <c r="B30" t="s">
         <v>138</v>
@@ -6492,7 +7359,7 @@
         <v>44</v>
       </c>
       <c r="D30" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E30" t="s">
         <v>8</v>
@@ -6515,16 +7382,16 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>312</v>
+        <v>367</v>
       </c>
       <c r="B31" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
       </c>
       <c r="D31" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E31" t="s">
         <v>8</v>
@@ -6565,7 +7432,7 @@
         <v>8</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>313</v>
+        <v>368</v>
       </c>
       <c r="H32" t="s">
         <v>8</v>
@@ -6582,13 +7449,13 @@
         <v>58</v>
       </c>
       <c r="B33" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C33" t="s">
         <v>8</v>
       </c>
       <c r="D33" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E33" t="s">
         <v>8</v>
@@ -6611,16 +7478,16 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>314</v>
+        <v>369</v>
       </c>
       <c r="B34" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C34" t="s">
         <v>8</v>
       </c>
       <c r="D34" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E34" t="s">
         <v>8</v>
@@ -6643,7 +7510,7 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>315</v>
+        <v>370</v>
       </c>
       <c r="B35" t="s">
         <v>138</v>
@@ -6652,7 +7519,7 @@
         <v>171</v>
       </c>
       <c r="D35" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
@@ -6675,16 +7542,16 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>316</v>
+        <v>371</v>
       </c>
       <c r="B36" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C36" t="s">
         <v>8</v>
       </c>
       <c r="D36" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E36" t="s">
         <v>8</v>
@@ -6707,7 +7574,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>317</v>
+        <v>372</v>
       </c>
       <c r="B37" t="s">
         <v>138</v>
@@ -6716,7 +7583,7 @@
         <v>44</v>
       </c>
       <c r="D37" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E37" t="s">
         <v>8</v>
@@ -6739,16 +7606,16 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>317</v>
+        <v>372</v>
       </c>
       <c r="B38" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C38" t="s">
         <v>8</v>
       </c>
       <c r="D38" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E38" t="s">
         <v>8</v>
@@ -6771,7 +7638,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>318</v>
+        <v>373</v>
       </c>
       <c r="B39" t="s">
         <v>138</v>
@@ -6789,7 +7656,7 @@
         <v>8</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>319</v>
+        <v>374</v>
       </c>
       <c r="H39" t="s">
         <v>8</v>
@@ -6803,16 +7670,16 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>318</v>
+        <v>373</v>
       </c>
       <c r="B40" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C40" t="s">
         <v>8</v>
       </c>
       <c r="D40" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E40" t="s">
         <v>8</v>
@@ -6838,7 +7705,7 @@
         <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C41" t="s">
         <v>8</v>
@@ -6853,7 +7720,7 @@
         <v>8</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>321</v>
+        <v>376</v>
       </c>
       <c r="H41" t="s">
         <v>8</v>
@@ -6867,7 +7734,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>322</v>
+        <v>377</v>
       </c>
       <c r="B42" t="s">
         <v>138</v>
@@ -6876,7 +7743,7 @@
         <v>171</v>
       </c>
       <c r="D42" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E42" t="s">
         <v>8</v>
@@ -6899,16 +7766,16 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>323</v>
+        <v>378</v>
       </c>
       <c r="B43" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C43" t="s">
         <v>8</v>
       </c>
       <c r="D43" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E43" t="s">
         <v>8</v>
@@ -6931,7 +7798,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="B44" t="s">
         <v>138</v>
@@ -6940,7 +7807,7 @@
         <v>44</v>
       </c>
       <c r="D44" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E44" t="s">
         <v>8</v>
@@ -6963,16 +7830,16 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>324</v>
+        <v>379</v>
       </c>
       <c r="B45" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C45" t="s">
         <v>8</v>
       </c>
       <c r="D45" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E45" t="s">
         <v>8</v>
@@ -6995,7 +7862,7 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
       <c r="B46" t="s">
         <v>138</v>
@@ -7013,7 +7880,7 @@
         <v>8</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>326</v>
+        <v>381</v>
       </c>
       <c r="H46" t="s">
         <v>8</v>
@@ -7027,16 +7894,16 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
       <c r="B47" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C47" t="s">
         <v>8</v>
       </c>
       <c r="D47" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E47" t="s">
         <v>8</v>
@@ -7059,16 +7926,16 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>327</v>
+        <v>382</v>
       </c>
       <c r="B48" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C48" t="s">
         <v>8</v>
       </c>
       <c r="D48" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E48" t="s">
         <v>8</v>
@@ -7091,16 +7958,16 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>328</v>
+        <v>383</v>
       </c>
       <c r="B49" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C49" t="s">
         <v>8</v>
       </c>
       <c r="D49" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E49" t="s">
         <v>8</v>
@@ -7123,7 +7990,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>329</v>
+        <v>384</v>
       </c>
       <c r="B50" t="s">
         <v>138</v>
@@ -7132,7 +7999,7 @@
         <v>168</v>
       </c>
       <c r="D50" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E50" t="s">
         <v>8</v>
@@ -7155,16 +8022,16 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>329</v>
+        <v>384</v>
       </c>
       <c r="B51" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C51" t="s">
         <v>8</v>
       </c>
       <c r="D51" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E51" t="s">
         <v>8</v>
@@ -7187,7 +8054,7 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>330</v>
+        <v>385</v>
       </c>
       <c r="B52" t="s">
         <v>138</v>
@@ -7196,7 +8063,7 @@
         <v>166</v>
       </c>
       <c r="D52" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E52" t="s">
         <v>8</v>
@@ -7219,16 +8086,16 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>330</v>
+        <v>385</v>
       </c>
       <c r="B53" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C53" t="s">
         <v>8</v>
       </c>
       <c r="D53" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E53" t="s">
         <v>8</v>
@@ -7251,16 +8118,16 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>331</v>
+        <v>386</v>
       </c>
       <c r="B54" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C54" t="s">
         <v>8</v>
       </c>
       <c r="D54" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E54" t="s">
         <v>8</v>
@@ -7283,16 +8150,16 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>332</v>
+        <v>387</v>
       </c>
       <c r="B55" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C55" t="s">
         <v>8</v>
       </c>
       <c r="D55" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E55" t="s">
         <v>8</v>
@@ -7315,7 +8182,7 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>333</v>
+        <v>388</v>
       </c>
       <c r="B56" t="s">
         <v>138</v>
@@ -7347,7 +8214,7 @@
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>334</v>
+        <v>389</v>
       </c>
       <c r="B57" t="s">
         <v>138</v>
@@ -7356,7 +8223,7 @@
         <v>168</v>
       </c>
       <c r="D57" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E57" t="s">
         <v>8</v>
@@ -7379,7 +8246,7 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>335</v>
+        <v>390</v>
       </c>
       <c r="B58" t="s">
         <v>138</v>
@@ -7388,7 +8255,7 @@
         <v>166</v>
       </c>
       <c r="D58" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E58" t="s">
         <v>8</v>
@@ -7411,16 +8278,16 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>335</v>
+        <v>390</v>
       </c>
       <c r="B59" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C59" t="s">
         <v>8</v>
       </c>
       <c r="D59" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E59" t="s">
         <v>8</v>
@@ -7443,16 +8310,16 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="B60" t="s">
         <v>336</v>
       </c>
-      <c r="B60" t="s">
-        <v>281</v>
-      </c>
       <c r="C60" t="s">
         <v>8</v>
       </c>
       <c r="D60" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E60" t="s">
         <v>8</v>
@@ -7475,7 +8342,7 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>337</v>
+        <v>392</v>
       </c>
       <c r="B61" t="s">
         <v>138</v>
@@ -7507,7 +8374,7 @@
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>338</v>
+        <v>393</v>
       </c>
       <c r="B62" t="s">
         <v>138</v>
@@ -7516,7 +8383,7 @@
         <v>168</v>
       </c>
       <c r="D62" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E62" t="s">
         <v>8</v>
@@ -7539,16 +8406,16 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>338</v>
+        <v>393</v>
       </c>
       <c r="B63" t="s">
-        <v>281</v>
+        <v>336</v>
       </c>
       <c r="C63" t="s">
         <v>8</v>
       </c>
       <c r="D63" t="s">
-        <v>286</v>
+        <v>341</v>
       </c>
       <c r="E63" t="s">
         <v>8</v>
@@ -7571,7 +8438,7 @@
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>339</v>
+        <v>394</v>
       </c>
       <c r="B64" t="s">
         <v>138</v>
@@ -7580,7 +8447,7 @@
         <v>166</v>
       </c>
       <c r="D64" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E64" t="s">
         <v>8</v>
@@ -7603,16 +8470,16 @@
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="B65" t="s">
+        <v>336</v>
+      </c>
+      <c r="C65" t="s">
+        <v>8</v>
+      </c>
+      <c r="D65" t="s">
         <v>339</v>
-      </c>
-      <c r="B65" t="s">
-        <v>281</v>
-      </c>
-      <c r="C65" t="s">
-        <v>8</v>
-      </c>
-      <c r="D65" t="s">
-        <v>284</v>
       </c>
       <c r="E65" t="s">
         <v>8</v>
@@ -7635,7 +8502,7 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>340</v>
+        <v>395</v>
       </c>
       <c r="B66" t="s">
         <v>138</v>
@@ -7667,7 +8534,7 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>341</v>
+        <v>396</v>
       </c>
       <c r="B67" t="s">
         <v>138</v>
@@ -7676,7 +8543,7 @@
         <v>171</v>
       </c>
       <c r="D67" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E67" t="s">
         <v>8</v>
@@ -7699,7 +8566,7 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>342</v>
+        <v>397</v>
       </c>
       <c r="B68" t="s">
         <v>138</v>
@@ -7708,7 +8575,7 @@
         <v>168</v>
       </c>
       <c r="D68" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E68" t="s">
         <v>8</v>
@@ -7731,7 +8598,7 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>343</v>
+        <v>398</v>
       </c>
       <c r="B69" t="s">
         <v>138</v>
@@ -7740,7 +8607,7 @@
         <v>44</v>
       </c>
       <c r="D69" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E69" t="s">
         <v>8</v>
@@ -7763,7 +8630,7 @@
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>344</v>
+        <v>399</v>
       </c>
       <c r="B70" t="s">
         <v>138</v>
@@ -7772,7 +8639,7 @@
         <v>171</v>
       </c>
       <c r="D70" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E70" t="s">
         <v>8</v>
@@ -7795,7 +8662,7 @@
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>345</v>
+        <v>400</v>
       </c>
       <c r="B71" t="s">
         <v>138</v>
@@ -7804,7 +8671,7 @@
         <v>168</v>
       </c>
       <c r="D71" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E71" t="s">
         <v>8</v>
@@ -7827,7 +8694,7 @@
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>346</v>
+        <v>401</v>
       </c>
       <c r="B72" t="s">
         <v>138</v>
@@ -7836,7 +8703,7 @@
         <v>44</v>
       </c>
       <c r="D72" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E72" t="s">
         <v>8</v>
@@ -7859,10 +8726,10 @@
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>347</v>
+        <v>402</v>
       </c>
       <c r="B73" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C73" t="s">
         <v>8</v>
@@ -7877,7 +8744,7 @@
         <v>8</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>348</v>
+        <v>403</v>
       </c>
       <c r="H73" t="s">
         <v>8</v>
@@ -7891,7 +8758,7 @@
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>349</v>
+        <v>404</v>
       </c>
       <c r="B74" t="s">
         <v>138</v>
@@ -7900,7 +8767,7 @@
         <v>171</v>
       </c>
       <c r="D74" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E74" t="s">
         <v>8</v>
@@ -7923,7 +8790,7 @@
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>350</v>
+        <v>405</v>
       </c>
       <c r="B75" t="s">
         <v>138</v>
@@ -7932,7 +8799,7 @@
         <v>168</v>
       </c>
       <c r="D75" t="s">
-        <v>279</v>
+        <v>334</v>
       </c>
       <c r="E75" t="s">
         <v>8</v>
@@ -7955,7 +8822,7 @@
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>351</v>
+        <v>406</v>
       </c>
       <c r="B76" t="s">
         <v>138</v>
@@ -7964,7 +8831,7 @@
         <v>44</v>
       </c>
       <c r="D76" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E76" t="s">
         <v>8</v>
@@ -7987,7 +8854,7 @@
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>352</v>
+        <v>407</v>
       </c>
       <c r="B77" t="s">
         <v>138</v>
@@ -7996,7 +8863,7 @@
         <v>166</v>
       </c>
       <c r="D77" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E77" t="s">
         <v>8</v>
@@ -8019,7 +8886,7 @@
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>353</v>
+        <v>408</v>
       </c>
       <c r="B78" t="s">
         <v>138</v>
@@ -8028,7 +8895,7 @@
         <v>171</v>
       </c>
       <c r="D78" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E78" t="s">
         <v>8</v>
@@ -8051,7 +8918,7 @@
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>354</v>
+        <v>409</v>
       </c>
       <c r="B79" t="s">
         <v>138</v>
@@ -8060,7 +8927,7 @@
         <v>72</v>
       </c>
       <c r="D79" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="E79" t="s">
         <v>8</v>
@@ -8083,7 +8950,7 @@
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>356</v>
+        <v>411</v>
       </c>
       <c r="B80" t="s">
         <v>138</v>
@@ -8092,7 +8959,7 @@
         <v>171</v>
       </c>
       <c r="D80" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E80" t="s">
         <v>8</v>
@@ -8115,7 +8982,7 @@
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>357</v>
+        <v>412</v>
       </c>
       <c r="B81" t="s">
         <v>138</v>
@@ -8124,7 +8991,7 @@
         <v>166</v>
       </c>
       <c r="D81" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E81" t="s">
         <v>8</v>
@@ -8147,7 +9014,7 @@
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>358</v>
+        <v>413</v>
       </c>
       <c r="B82" t="s">
         <v>138</v>
@@ -8156,7 +9023,7 @@
         <v>72</v>
       </c>
       <c r="D82" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="E82" t="s">
         <v>8</v>
@@ -8179,10 +9046,10 @@
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>359</v>
+        <v>414</v>
       </c>
       <c r="B83" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C83" t="s">
         <v>8</v>
@@ -8197,7 +9064,7 @@
         <v>8</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>321</v>
+        <v>376</v>
       </c>
       <c r="H83" t="s">
         <v>8</v>
@@ -8211,7 +9078,7 @@
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>360</v>
+        <v>415</v>
       </c>
       <c r="B84" t="s">
         <v>138</v>
@@ -8220,7 +9087,7 @@
         <v>166</v>
       </c>
       <c r="D84" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E84" t="s">
         <v>8</v>
@@ -8243,7 +9110,7 @@
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>361</v>
+        <v>416</v>
       </c>
       <c r="B85" t="s">
         <v>138</v>
@@ -8252,7 +9119,7 @@
         <v>171</v>
       </c>
       <c r="D85" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E85" t="s">
         <v>8</v>
@@ -8275,7 +9142,7 @@
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>362</v>
+        <v>417</v>
       </c>
       <c r="B86" t="s">
         <v>138</v>
@@ -8284,7 +9151,7 @@
         <v>72</v>
       </c>
       <c r="D86" t="s">
-        <v>355</v>
+        <v>410</v>
       </c>
       <c r="E86" t="s">
         <v>8</v>
@@ -8307,7 +9174,7 @@
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>363</v>
+        <v>418</v>
       </c>
       <c r="B87" t="s">
         <v>138</v>
@@ -8316,7 +9183,7 @@
         <v>166</v>
       </c>
       <c r="D87" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E87" t="s">
         <v>8</v>
@@ -8339,7 +9206,7 @@
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>364</v>
+        <v>419</v>
       </c>
       <c r="B88" t="s">
         <v>138</v>
@@ -8348,7 +9215,7 @@
         <v>44</v>
       </c>
       <c r="D88" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E88" t="s">
         <v>8</v>
@@ -8371,7 +9238,7 @@
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>365</v>
+        <v>420</v>
       </c>
       <c r="B89" t="s">
         <v>138</v>
@@ -8380,7 +9247,7 @@
         <v>166</v>
       </c>
       <c r="D89" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E89" t="s">
         <v>8</v>
@@ -8403,7 +9270,7 @@
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>366</v>
+        <v>421</v>
       </c>
       <c r="B90" t="s">
         <v>138</v>
@@ -8412,7 +9279,7 @@
         <v>44</v>
       </c>
       <c r="D90" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E90" t="s">
         <v>8</v>
@@ -8435,7 +9302,7 @@
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>367</v>
+        <v>422</v>
       </c>
       <c r="B91" t="s">
         <v>138</v>
@@ -8444,7 +9311,7 @@
         <v>166</v>
       </c>
       <c r="D91" t="s">
-        <v>290</v>
+        <v>345</v>
       </c>
       <c r="E91" t="s">
         <v>8</v>
@@ -8467,7 +9334,7 @@
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>368</v>
+        <v>423</v>
       </c>
       <c r="B92" t="s">
         <v>138</v>
@@ -8476,7 +9343,7 @@
         <v>44</v>
       </c>
       <c r="D92" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E92" t="s">
         <v>8</v>
@@ -8499,7 +9366,7 @@
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>369</v>
+        <v>424</v>
       </c>
       <c r="B93" t="s">
         <v>138</v>
@@ -8508,7 +9375,7 @@
         <v>44</v>
       </c>
       <c r="D93" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E93" t="s">
         <v>8</v>
@@ -8531,7 +9398,7 @@
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>370</v>
+        <v>425</v>
       </c>
       <c r="B94" t="s">
         <v>138</v>
@@ -8540,7 +9407,7 @@
         <v>166</v>
       </c>
       <c r="D94" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E94" t="s">
         <v>8</v>
@@ -8563,10 +9430,10 @@
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>371</v>
+        <v>426</v>
       </c>
       <c r="B95" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C95" t="s">
         <v>8</v>
@@ -8581,7 +9448,7 @@
         <v>8</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>321</v>
+        <v>376</v>
       </c>
       <c r="H95" t="s">
         <v>8</v>
@@ -8595,7 +9462,7 @@
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>372</v>
+        <v>427</v>
       </c>
       <c r="B96" t="s">
         <v>138</v>
@@ -8604,7 +9471,7 @@
         <v>72</v>
       </c>
       <c r="D96" t="s">
-        <v>373</v>
+        <v>428</v>
       </c>
       <c r="E96" t="s">
         <v>8</v>
@@ -8627,7 +9494,7 @@
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>374</v>
+        <v>429</v>
       </c>
       <c r="B97" t="s">
         <v>138</v>
@@ -8636,7 +9503,7 @@
         <v>44</v>
       </c>
       <c r="D97" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E97" t="s">
         <v>8</v>
@@ -8659,7 +9526,7 @@
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>375</v>
+        <v>430</v>
       </c>
       <c r="B98" t="s">
         <v>138</v>
@@ -8668,7 +9535,7 @@
         <v>166</v>
       </c>
       <c r="D98" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E98" t="s">
         <v>8</v>
@@ -8691,7 +9558,7 @@
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>376</v>
+        <v>431</v>
       </c>
       <c r="B99" t="s">
         <v>138</v>
@@ -8700,7 +9567,7 @@
         <v>72</v>
       </c>
       <c r="D99" t="s">
-        <v>373</v>
+        <v>428</v>
       </c>
       <c r="E99" t="s">
         <v>8</v>
@@ -8723,10 +9590,10 @@
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>377</v>
+        <v>432</v>
       </c>
       <c r="B100" t="s">
-        <v>320</v>
+        <v>375</v>
       </c>
       <c r="C100" t="s">
         <v>8</v>
@@ -8741,7 +9608,7 @@
         <v>8</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>378</v>
+        <v>433</v>
       </c>
       <c r="H100" t="s">
         <v>8</v>
@@ -8755,7 +9622,7 @@
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>379</v>
+        <v>434</v>
       </c>
       <c r="B101" t="s">
         <v>138</v>
@@ -8764,7 +9631,7 @@
         <v>44</v>
       </c>
       <c r="D101" t="s">
-        <v>282</v>
+        <v>337</v>
       </c>
       <c r="E101" t="s">
         <v>8</v>
@@ -8787,7 +9654,7 @@
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
-        <v>380</v>
+        <v>435</v>
       </c>
       <c r="B102" t="s">
         <v>138</v>
@@ -8796,7 +9663,7 @@
         <v>166</v>
       </c>
       <c r="D102" t="s">
-        <v>288</v>
+        <v>343</v>
       </c>
       <c r="E102" t="s">
         <v>8</v>
@@ -8819,7 +9686,7 @@
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
-        <v>381</v>
+        <v>436</v>
       </c>
       <c r="B103" t="s">
         <v>138</v>
@@ -8828,7 +9695,7 @@
         <v>72</v>
       </c>
       <c r="D103" t="s">
-        <v>373</v>
+        <v>428</v>
       </c>
       <c r="E103" t="s">
         <v>8</v>
@@ -8851,7 +9718,7 @@
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
-        <v>382</v>
+        <v>437</v>
       </c>
       <c r="B104" t="s">
         <v>138</v>
@@ -8860,7 +9727,7 @@
         <v>171</v>
       </c>
       <c r="D104" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E104" t="s">
         <v>8</v>
@@ -8883,7 +9750,7 @@
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
-        <v>383</v>
+        <v>438</v>
       </c>
       <c r="B105" t="s">
         <v>138</v>
@@ -8892,7 +9759,7 @@
         <v>44</v>
       </c>
       <c r="D105" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E105" t="s">
         <v>8</v>
@@ -8915,7 +9782,7 @@
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
-        <v>384</v>
+        <v>439</v>
       </c>
       <c r="B106" t="s">
         <v>138</v>
@@ -8924,7 +9791,7 @@
         <v>171</v>
       </c>
       <c r="D106" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E106" t="s">
         <v>8</v>
@@ -8947,7 +9814,7 @@
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
-        <v>385</v>
+        <v>440</v>
       </c>
       <c r="B107" t="s">
         <v>138</v>
@@ -8956,7 +9823,7 @@
         <v>44</v>
       </c>
       <c r="D107" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E107" t="s">
         <v>8</v>
@@ -8979,7 +9846,7 @@
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
-        <v>386</v>
+        <v>441</v>
       </c>
       <c r="B108" t="s">
         <v>138</v>
@@ -8988,7 +9855,7 @@
         <v>171</v>
       </c>
       <c r="D108" t="s">
-        <v>310</v>
+        <v>365</v>
       </c>
       <c r="E108" t="s">
         <v>8</v>
@@ -9011,7 +9878,7 @@
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
-        <v>387</v>
+        <v>442</v>
       </c>
       <c r="B109" t="s">
         <v>138</v>
@@ -9020,7 +9887,7 @@
         <v>44</v>
       </c>
       <c r="D109" t="s">
-        <v>284</v>
+        <v>339</v>
       </c>
       <c r="E109" t="s">
         <v>8</v>

</xml_diff>